<commit_message>
fix: carga de usuario en excel
</commit_message>
<xml_diff>
--- a/deposito.xlsx
+++ b/deposito.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEP1A44502</t>
+          <t>DEP1C32202</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,12 +462,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -476,6 +476,38 @@
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DEP1C43301</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DEP1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
@@ -492,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,41 +545,138 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DEP1A44502</t>
+          <t>DEP1C32202</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>adfd456</t>
+          <t>dpso345</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DEP1A44502</t>
+          <t>DEP1C32202</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>adps567</t>
+          <t>fpro459</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DEP1A44502</t>
+          <t>DEP1C32202</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>dfsp321</t>
+          <t>zwwo322</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DEP1C32202</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dpyo987</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DEP1C43301</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ddos212</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DEP1C43301</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ppfg553</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DEP1C43301</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>dovv123</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pancho1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DEP1C43301</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fcof443</t>
         </is>
       </c>
     </row>

</xml_diff>